<commit_message>
Daily NSE scan: 2026-09-15
</commit_message>
<xml_diff>
--- a/output/2026-09-15/enriched_analysis.xlsx
+++ b/output/2026-09-15/enriched_analysis.xlsx
@@ -813,10 +813,10 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>3.66</v>
+        <v>3.653</v>
       </c>
       <c r="Q2" t="n">
-        <v>2894</v>
+        <v>2899</v>
       </c>
       <c r="R2" t="n">
         <v>22.7</v>
@@ -995,13 +995,13 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>0.08</v>
+        <v>0.079</v>
       </c>
       <c r="Q3" t="n">
-        <v>2661</v>
+        <v>2691</v>
       </c>
       <c r="R3" t="n">
-        <v>9.140000000000001</v>
+        <v>9.27</v>
       </c>
       <c r="S3" t="n">
         <v>36</v>
@@ -1177,13 +1177,13 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>0.133</v>
+        <v>0.134</v>
       </c>
       <c r="Q4" t="n">
-        <v>2364</v>
+        <v>2342</v>
       </c>
       <c r="R4" t="n">
-        <v>20.8</v>
+        <v>20.5</v>
       </c>
       <c r="S4" t="n">
         <v>-3</v>
@@ -1541,13 +1541,13 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>0.885</v>
+        <v>0.877</v>
       </c>
       <c r="Q6" t="n">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="R6" t="n">
-        <v>8.890000000000001</v>
+        <v>8.970000000000001</v>
       </c>
       <c r="S6" t="n">
         <v>17</v>
@@ -1723,10 +1723,10 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>2.814</v>
+        <v>2.803</v>
       </c>
       <c r="Q7" t="n">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="R7" t="n">
         <v>11.6</v>
@@ -1905,13 +1905,13 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>0.058</v>
+        <v>0.061</v>
       </c>
       <c r="Q8" t="n">
-        <v>1418</v>
+        <v>1343</v>
       </c>
       <c r="R8" t="n">
-        <v>19.1</v>
+        <v>18.1</v>
       </c>
       <c r="S8" t="n">
         <v>55</v>
@@ -2087,10 +2087,10 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>0.638</v>
+        <v>0.645</v>
       </c>
       <c r="Q9" t="n">
-        <v>334</v>
+        <v>330</v>
       </c>
       <c r="R9" t="inlineStr"/>
       <c r="S9" t="n">
@@ -2267,13 +2267,13 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>0.323</v>
+        <v>0.324</v>
       </c>
       <c r="Q10" t="n">
-        <v>2629</v>
+        <v>2617</v>
       </c>
       <c r="R10" t="n">
-        <v>21.5</v>
+        <v>21.4</v>
       </c>
       <c r="S10" t="n">
         <v>8</v>
@@ -2449,10 +2449,10 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>2.282</v>
+        <v>2.285</v>
       </c>
       <c r="Q11" t="n">
-        <v>2611</v>
+        <v>2608</v>
       </c>
       <c r="R11" t="n">
         <v>205</v>
@@ -2634,10 +2634,10 @@
         <v>0.046</v>
       </c>
       <c r="Q12" t="n">
-        <v>15522</v>
+        <v>15611</v>
       </c>
       <c r="R12" t="n">
-        <v>39.5</v>
+        <v>39.7</v>
       </c>
       <c r="S12" t="n">
         <v>83</v>
@@ -2813,13 +2813,13 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>0.149</v>
+        <v>0.15</v>
       </c>
       <c r="Q13" t="n">
-        <v>743</v>
+        <v>740</v>
       </c>
       <c r="R13" t="n">
-        <v>62.1</v>
+        <v>61.8</v>
       </c>
       <c r="S13" t="n">
         <v>3</v>
@@ -3178,10 +3178,10 @@
         <v>0.194</v>
       </c>
       <c r="Q15" t="n">
-        <v>894</v>
+        <v>890</v>
       </c>
       <c r="R15" t="n">
-        <v>8.779999999999999</v>
+        <v>8.74</v>
       </c>
       <c r="S15" t="n">
         <v>7</v>
@@ -3360,10 +3360,10 @@
         <v>0.013</v>
       </c>
       <c r="Q16" t="n">
-        <v>16119</v>
+        <v>16130</v>
       </c>
       <c r="R16" t="n">
-        <v>20.4</v>
+        <v>20.5</v>
       </c>
       <c r="S16" t="n">
         <v>16</v>
@@ -3539,13 +3539,13 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>0.397</v>
+        <v>0.411</v>
       </c>
       <c r="Q17" t="n">
-        <v>1138</v>
+        <v>1099</v>
       </c>
       <c r="R17" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="S17" t="n">
         <v>21</v>
@@ -3721,13 +3721,13 @@
         </is>
       </c>
       <c r="P18" t="n">
-        <v>0.537</v>
+        <v>0.532</v>
       </c>
       <c r="Q18" t="n">
-        <v>391</v>
+        <v>395</v>
       </c>
       <c r="R18" t="n">
-        <v>1261</v>
+        <v>1274</v>
       </c>
       <c r="S18" t="n">
         <v>-61</v>
@@ -3899,10 +3899,10 @@
         </is>
       </c>
       <c r="P19" t="n">
-        <v>1.612</v>
+        <v>1.7</v>
       </c>
       <c r="Q19" t="n">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="R19" t="inlineStr"/>
       <c r="S19" t="n">
@@ -4079,13 +4079,13 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>0.096</v>
+        <v>0.095</v>
       </c>
       <c r="Q20" t="n">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="R20" t="n">
-        <v>29</v>
+        <v>29.5</v>
       </c>
       <c r="S20" t="n">
         <v>24</v>
@@ -4396,7 +4396,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>PNGS REVA DIAMOND JEWELLERY LIMITED</t>
+          <t>PNGS Reva Diamond Jewellery Limited</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -4443,13 +4443,13 @@
         </is>
       </c>
       <c r="P22" t="n">
-        <v>0.112</v>
+        <v>0.111</v>
       </c>
       <c r="Q22" t="n">
-        <v>1558</v>
+        <v>1574</v>
       </c>
       <c r="R22" t="n">
-        <v>18.4</v>
+        <v>18.6</v>
       </c>
       <c r="S22" t="n">
         <v>581</v>
@@ -4623,10 +4623,10 @@
         </is>
       </c>
       <c r="P23" t="n">
-        <v>1.082</v>
+        <v>1.081</v>
       </c>
       <c r="Q23" t="n">
-        <v>9494</v>
+        <v>9503</v>
       </c>
       <c r="R23" t="n">
         <v>12.5</v>
@@ -4805,13 +4805,13 @@
         </is>
       </c>
       <c r="P24" t="n">
-        <v>0.132</v>
+        <v>0.134</v>
       </c>
       <c r="Q24" t="n">
-        <v>380</v>
+        <v>374</v>
       </c>
       <c r="R24" t="n">
-        <v>6.14</v>
+        <v>6.04</v>
       </c>
       <c r="S24" t="n">
         <v>118</v>
@@ -4983,13 +4983,13 @@
         </is>
       </c>
       <c r="P25" t="n">
-        <v>0.2</v>
+        <v>0.198</v>
       </c>
       <c r="Q25" t="n">
-        <v>854</v>
+        <v>864</v>
       </c>
       <c r="R25" t="n">
-        <v>24.4</v>
+        <v>24.8</v>
       </c>
       <c r="S25" t="n">
         <v>19</v>
@@ -5165,13 +5165,13 @@
         </is>
       </c>
       <c r="P26" t="n">
-        <v>0.056</v>
+        <v>0.055</v>
       </c>
       <c r="Q26" t="n">
-        <v>1960</v>
+        <v>1986</v>
       </c>
       <c r="R26" t="n">
-        <v>45</v>
+        <v>45.6</v>
       </c>
       <c r="S26" t="n">
         <v>20</v>
@@ -5350,10 +5350,10 @@
         <v>0.038</v>
       </c>
       <c r="Q27" t="n">
-        <v>3542</v>
+        <v>3529</v>
       </c>
       <c r="R27" t="n">
-        <v>21</v>
+        <v>20.9</v>
       </c>
       <c r="S27" t="n">
         <v>-4</v>
@@ -5714,10 +5714,10 @@
         <v>0.007</v>
       </c>
       <c r="Q29" t="n">
-        <v>5632</v>
+        <v>5640</v>
       </c>
       <c r="R29" t="n">
-        <v>9.51</v>
+        <v>9.529999999999999</v>
       </c>
       <c r="S29" t="n">
         <v>43</v>
@@ -5893,13 +5893,13 @@
         </is>
       </c>
       <c r="P30" t="n">
-        <v>0.199</v>
+        <v>0.201</v>
       </c>
       <c r="Q30" t="n">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="R30" t="n">
-        <v>26.9</v>
+        <v>26.7</v>
       </c>
       <c r="S30" t="n">
         <v>21</v>
@@ -6075,13 +6075,13 @@
         </is>
       </c>
       <c r="P31" t="n">
-        <v>0.502</v>
+        <v>0.507</v>
       </c>
       <c r="Q31" t="n">
-        <v>677</v>
+        <v>671</v>
       </c>
       <c r="R31" t="n">
-        <v>14.9</v>
+        <v>14.8</v>
       </c>
       <c r="S31" t="n">
         <v>-1</v>
@@ -6257,13 +6257,13 @@
         </is>
       </c>
       <c r="P32" t="n">
-        <v>0.594</v>
+        <v>0.598</v>
       </c>
       <c r="Q32" t="n">
-        <v>2298</v>
+        <v>2281</v>
       </c>
       <c r="R32" t="n">
-        <v>680</v>
+        <v>675</v>
       </c>
       <c r="S32" t="n">
         <v>3</v>
@@ -6439,13 +6439,13 @@
         </is>
       </c>
       <c r="P33" t="n">
-        <v>0.269</v>
+        <v>0.271</v>
       </c>
       <c r="Q33" t="n">
-        <v>1103</v>
+        <v>1095</v>
       </c>
       <c r="R33" t="n">
-        <v>19.6</v>
+        <v>19.5</v>
       </c>
       <c r="S33" t="n">
         <v>12</v>
@@ -6621,13 +6621,13 @@
         </is>
       </c>
       <c r="P34" t="n">
-        <v>0.047</v>
+        <v>0.046</v>
       </c>
       <c r="Q34" t="n">
-        <v>898</v>
+        <v>904</v>
       </c>
       <c r="R34" t="n">
-        <v>95.90000000000001</v>
+        <v>96.59999999999999</v>
       </c>
       <c r="S34" t="n">
         <v>15</v>
@@ -6803,13 +6803,13 @@
         </is>
       </c>
       <c r="P35" t="n">
-        <v>0.391</v>
+        <v>0.396</v>
       </c>
       <c r="Q35" t="n">
-        <v>409</v>
+        <v>404</v>
       </c>
       <c r="R35" t="n">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="S35" t="n">
         <v>246</v>
@@ -6988,7 +6988,7 @@
         <v>0.097</v>
       </c>
       <c r="Q36" t="n">
-        <v>1531</v>
+        <v>1530</v>
       </c>
       <c r="R36" t="n">
         <v>13.8</v>
@@ -7170,7 +7170,7 @@
         <v>0.008999999999999999</v>
       </c>
       <c r="Q37" t="n">
-        <v>53164</v>
+        <v>53053</v>
       </c>
       <c r="R37" t="n">
         <v>45</v>
@@ -7297,12 +7297,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>TAINWALCHM</t>
+          <t>SGIL</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>TAINWALA CHEMICALS AND PLASTICS (INDIA) LIMITED</t>
+          <t>SYNERGY GREEN INDUSTRIES LIMITED</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -7314,87 +7314,85 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F38" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="G38" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="H38" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="I38" t="n">
-        <v>207.79</v>
+        <v>592.2</v>
       </c>
       <c r="J38" t="n">
-        <v>210.84</v>
+        <v>593.62</v>
       </c>
       <c r="K38" t="n">
-        <v>-1.4</v>
+        <v>-0.2</v>
       </c>
       <c r="L38" t="n">
-        <v>67.04000000000001</v>
+        <v>74.02</v>
       </c>
       <c r="M38" t="n">
-        <v>0.42</v>
+        <v>0.25</v>
       </c>
       <c r="N38" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>10-09-2026</t>
+          <t>11-09-2026</t>
         </is>
       </c>
       <c r="P38" t="n">
-        <v>0.21</v>
+        <v>0.027</v>
       </c>
       <c r="Q38" t="n">
-        <v>200</v>
-      </c>
-      <c r="R38" t="n">
-        <v>24.9</v>
-      </c>
+        <v>928</v>
+      </c>
+      <c r="R38" t="inlineStr"/>
       <c r="S38" t="n">
-        <v>12</v>
+        <v>-2</v>
       </c>
       <c r="T38" t="n">
-        <v>0.03</v>
+        <v>5</v>
       </c>
       <c r="U38" t="n">
-        <v>16</v>
+        <v>-152</v>
       </c>
       <c r="V38" t="n">
-        <v>0.03</v>
+        <v>-6.5</v>
       </c>
       <c r="W38" t="n">
-        <v>7.91</v>
+        <v>9.24</v>
       </c>
       <c r="X38" t="n">
-        <v>0</v>
+        <v>2.23</v>
       </c>
       <c r="Y38" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z38" t="n">
-        <v>3.16</v>
+        <v>6</v>
       </c>
       <c r="AA38" t="n">
-        <v>208.64</v>
+        <v>590.46</v>
       </c>
       <c r="AB38" t="n">
-        <v>195.46</v>
+        <v>545.01</v>
       </c>
       <c r="AC38" t="n">
-        <v>2.1</v>
+        <v>17.9</v>
       </c>
       <c r="AD38" t="n">
-        <v>210.8429673885985</v>
+        <v>593.6235208886742</v>
       </c>
       <c r="AE38" t="n">
-        <v>-1.4</v>
+        <v>-0.2</v>
       </c>
       <c r="AF38" t="inlineStr">
         <is>
@@ -7403,92 +7401,92 @@
       </c>
       <c r="AG38" t="inlineStr">
         <is>
-          <t>Confirmed Accumulation</t>
+          <t>Early Accumulation</t>
         </is>
       </c>
       <c r="AH38" t="inlineStr">
         <is>
-          <t>Confirmed Accumulation</t>
+          <t>Early Accumulation</t>
         </is>
       </c>
       <c r="AI38" t="inlineStr">
         <is>
-          <t>18-08-2026</t>
+          <t>28-08-2026</t>
         </is>
       </c>
       <c r="AJ38" t="inlineStr">
         <is>
-          <t>10-09-2026</t>
+          <t>11-09-2026</t>
         </is>
       </c>
       <c r="AK38" t="n">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="AL38" t="n">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="AM38" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AN38" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO38" t="n">
         <v>2</v>
       </c>
-      <c r="AO38" t="n">
-        <v>4</v>
-      </c>
       <c r="AP38" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="AQ38" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="AR38" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="AS38" t="n">
-        <v>1087797</v>
+        <v>322003</v>
       </c>
       <c r="AT38" t="n">
-        <v>1371280</v>
+        <v>1288195</v>
       </c>
       <c r="AU38" t="n">
-        <v>4234781</v>
+        <v>2458195</v>
       </c>
       <c r="AV38" t="n">
-        <v>4234781</v>
+        <v>2458195</v>
       </c>
       <c r="AW38" t="n">
-        <v>4234781</v>
+        <v>2458195</v>
       </c>
       <c r="AX38" t="n">
-        <v>1087797</v>
+        <v>322003</v>
       </c>
       <c r="AY38" t="n">
-        <v>4234781</v>
+        <v>2458195</v>
       </c>
       <c r="AZ38" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BA38" t="n">
         <v>0</v>
       </c>
       <c r="BB38" t="n">
-        <v>0.2569</v>
+        <v>0.131</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>HCLTECH</t>
+          <t>TAINWALCHM</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>HCL Technologies Limited</t>
+          <t>TAINWALA CHEMICALS AND PLASTICS (INDIA) LIMITED</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -7496,157 +7494,157 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="F39" t="n">
-        <v>26</v>
+        <v>9</v>
       </c>
       <c r="G39" t="n">
+        <v>13</v>
+      </c>
+      <c r="H39" t="n">
+        <v>-1</v>
+      </c>
+      <c r="I39" t="n">
+        <v>207.79</v>
+      </c>
+      <c r="J39" t="n">
+        <v>210.84</v>
+      </c>
+      <c r="K39" t="n">
+        <v>-1.4</v>
+      </c>
+      <c r="L39" t="n">
+        <v>67.04000000000001</v>
+      </c>
+      <c r="M39" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="N39" t="n">
+        <v>9</v>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>10-09-2026</t>
+        </is>
+      </c>
+      <c r="P39" t="n">
+        <v>0.216</v>
+      </c>
+      <c r="Q39" t="n">
+        <v>194</v>
+      </c>
+      <c r="R39" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="S39" t="n">
+        <v>12</v>
+      </c>
+      <c r="T39" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="U39" t="n">
+        <v>16</v>
+      </c>
+      <c r="V39" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="W39" t="n">
+        <v>7.91</v>
+      </c>
+      <c r="X39" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y39" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z39" t="n">
+        <v>3.16</v>
+      </c>
+      <c r="AA39" t="n">
+        <v>208.64</v>
+      </c>
+      <c r="AB39" t="n">
+        <v>195.46</v>
+      </c>
+      <c r="AC39" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="AD39" t="n">
+        <v>210.8429673885985</v>
+      </c>
+      <c r="AE39" t="n">
+        <v>-1.4</v>
+      </c>
+      <c r="AF39" t="inlineStr">
+        <is>
+          <t>Fresh</t>
+        </is>
+      </c>
+      <c r="AG39" t="inlineStr">
+        <is>
+          <t>Confirmed Accumulation</t>
+        </is>
+      </c>
+      <c r="AH39" t="inlineStr">
+        <is>
+          <t>Confirmed Accumulation</t>
+        </is>
+      </c>
+      <c r="AI39" t="inlineStr">
+        <is>
+          <t>18-08-2026</t>
+        </is>
+      </c>
+      <c r="AJ39" t="inlineStr">
+        <is>
+          <t>10-09-2026</t>
+        </is>
+      </c>
+      <c r="AK39" t="n">
+        <v>23</v>
+      </c>
+      <c r="AL39" t="n">
+        <v>28</v>
+      </c>
+      <c r="AM39" t="n">
+        <v>5</v>
+      </c>
+      <c r="AN39" t="n">
+        <v>2</v>
+      </c>
+      <c r="AO39" t="n">
         <v>4</v>
       </c>
-      <c r="H39" t="n">
-        <v>0</v>
-      </c>
-      <c r="I39" t="n">
-        <v>1206.1</v>
-      </c>
-      <c r="J39" t="n">
-        <v>1104.34</v>
-      </c>
-      <c r="K39" t="n">
-        <v>9.199999999999999</v>
-      </c>
-      <c r="L39" t="n">
-        <v>60.82</v>
-      </c>
-      <c r="M39" t="n">
-        <v>5.22</v>
-      </c>
-      <c r="N39" t="n">
-        <v>1</v>
-      </c>
-      <c r="O39" t="inlineStr">
-        <is>
-          <t>12-06-2026</t>
-        </is>
-      </c>
-      <c r="P39" t="n">
-        <v>0.002</v>
-      </c>
-      <c r="Q39" t="n">
-        <v>346060</v>
-      </c>
-      <c r="R39" t="n">
-        <v>19</v>
-      </c>
-      <c r="S39" t="n">
-        <v>7</v>
-      </c>
-      <c r="T39" t="n">
-        <v>4158</v>
-      </c>
-      <c r="U39" t="n">
-        <v>44</v>
-      </c>
-      <c r="V39" t="n">
-        <v>25.89</v>
-      </c>
-      <c r="W39" t="n">
-        <v>53.4</v>
-      </c>
-      <c r="X39" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="Y39" t="b">
-        <v>1</v>
-      </c>
-      <c r="Z39" t="n">
-        <v>29</v>
-      </c>
-      <c r="AA39" t="n">
-        <v>1282.03</v>
-      </c>
-      <c r="AB39" t="n">
-        <v>1380.71</v>
-      </c>
-      <c r="AC39" t="n">
-        <v>-11.4</v>
-      </c>
-      <c r="AD39" t="n">
-        <v>1104.337889591841</v>
-      </c>
-      <c r="AE39" t="n">
-        <v>9.199999999999999</v>
-      </c>
-      <c r="AF39" t="inlineStr">
-        <is>
-          <t>Stale</t>
-        </is>
-      </c>
-      <c r="AG39" t="inlineStr">
-        <is>
-          <t>Stale Accumulation</t>
-        </is>
-      </c>
-      <c r="AH39" t="inlineStr">
-        <is>
-          <t>Late — Poor Entry</t>
-        </is>
-      </c>
-      <c r="AI39" t="inlineStr">
-        <is>
-          <t>12-06-2026</t>
-        </is>
-      </c>
-      <c r="AJ39" t="inlineStr">
-        <is>
-          <t>12-06-2026</t>
-        </is>
-      </c>
-      <c r="AK39" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL39" t="n">
-        <v>95</v>
-      </c>
-      <c r="AM39" t="n">
-        <v>95</v>
-      </c>
-      <c r="AN39" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO39" t="n">
-        <v>0</v>
-      </c>
       <c r="AP39" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="AQ39" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="AR39" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="AS39" t="n">
-        <v>0</v>
+        <v>1087797</v>
       </c>
       <c r="AT39" t="n">
-        <v>0</v>
+        <v>1371280</v>
       </c>
       <c r="AU39" t="n">
-        <v>0</v>
+        <v>4234781</v>
       </c>
       <c r="AV39" t="n">
-        <v>0</v>
+        <v>4234781</v>
       </c>
       <c r="AW39" t="n">
-        <v>0</v>
+        <v>4234781</v>
       </c>
       <c r="AX39" t="n">
-        <v>0</v>
+        <v>1087797</v>
       </c>
       <c r="AY39" t="n">
-        <v>0</v>
+        <v>4234781</v>
       </c>
       <c r="AZ39" t="n">
         <v>1</v>
@@ -7655,18 +7653,18 @@
         <v>0</v>
       </c>
       <c r="BB39" t="n">
-        <v>0</v>
+        <v>0.2569</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>MANINFRA</t>
+          <t>HCLTECH</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>MAN INFRACONSTRUCTION LIMITED</t>
+          <t>HCL Technologies Limited</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -7678,87 +7676,87 @@
         </is>
       </c>
       <c r="E40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F40" t="n">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="G40" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="H40" t="n">
         <v>0</v>
       </c>
       <c r="I40" t="n">
-        <v>126.87</v>
+        <v>1206.1</v>
       </c>
       <c r="J40" t="n">
-        <v>105.19</v>
+        <v>1104.34</v>
       </c>
       <c r="K40" t="n">
-        <v>20.6</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="L40" t="n">
-        <v>67.15000000000001</v>
+        <v>60.82</v>
       </c>
       <c r="M40" t="n">
-        <v>2.63</v>
+        <v>5.22</v>
       </c>
       <c r="N40" t="n">
         <v>1</v>
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>25-06-2026</t>
+          <t>12-06-2026</t>
         </is>
       </c>
       <c r="P40" t="n">
-        <v>0.052</v>
+        <v>0.002</v>
       </c>
       <c r="Q40" t="n">
-        <v>5010</v>
+        <v>346752</v>
       </c>
       <c r="R40" t="n">
-        <v>32.7</v>
+        <v>19</v>
       </c>
       <c r="S40" t="n">
-        <v>-25</v>
+        <v>7</v>
       </c>
       <c r="T40" t="n">
-        <v>71</v>
+        <v>4158</v>
       </c>
       <c r="U40" t="n">
-        <v>-11</v>
+        <v>44</v>
       </c>
       <c r="V40" t="n">
-        <v>1.48</v>
+        <v>25.89</v>
       </c>
       <c r="W40" t="n">
-        <v>10.7</v>
+        <v>53.4</v>
       </c>
       <c r="X40" t="n">
-        <v>0</v>
+        <v>0.04</v>
       </c>
       <c r="Y40" t="b">
         <v>1</v>
       </c>
       <c r="Z40" t="n">
-        <v>69</v>
+        <v>29</v>
       </c>
       <c r="AA40" t="n">
-        <v>109.5</v>
+        <v>1282.03</v>
       </c>
       <c r="AB40" t="n">
-        <v>112.05</v>
+        <v>1380.71</v>
       </c>
       <c r="AC40" t="n">
-        <v>27.3</v>
+        <v>-11.4</v>
       </c>
       <c r="AD40" t="n">
-        <v>105.19</v>
+        <v>1104.337889591841</v>
       </c>
       <c r="AE40" t="n">
-        <v>20.6</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="AF40" t="inlineStr">
         <is>
@@ -7777,22 +7775,22 @@
       </c>
       <c r="AI40" t="inlineStr">
         <is>
-          <t>25-06-2026</t>
+          <t>12-06-2026</t>
         </is>
       </c>
       <c r="AJ40" t="inlineStr">
         <is>
-          <t>25-06-2026</t>
+          <t>12-06-2026</t>
         </is>
       </c>
       <c r="AK40" t="n">
         <v>0</v>
       </c>
       <c r="AL40" t="n">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="AM40" t="n">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="AN40" t="n">
         <v>0</v>
@@ -7807,7 +7805,7 @@
         <v>0</v>
       </c>
       <c r="AR40" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AS40" t="n">
         <v>0</v>
@@ -7822,7 +7820,7 @@
         <v>0</v>
       </c>
       <c r="AW40" t="n">
-        <v>78892500</v>
+        <v>0</v>
       </c>
       <c r="AX40" t="n">
         <v>0</v>
@@ -7895,13 +7893,13 @@
         </is>
       </c>
       <c r="P41" t="n">
-        <v>0.038</v>
+        <v>0.037</v>
       </c>
       <c r="Q41" t="n">
-        <v>824</v>
+        <v>835</v>
       </c>
       <c r="R41" t="n">
-        <v>19.8</v>
+        <v>20</v>
       </c>
       <c r="S41" t="inlineStr"/>
       <c r="T41" t="n">
@@ -8017,27 +8015,27 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>SGIL</t>
+          <t>MANINFRA</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>SYNERGY GREEN INDUSTRIES LIMITED</t>
+          <t>MAN INFRACONSTRUCTION LIMITED</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Avoid</t>
+          <t>Fundamental Watch</t>
         </is>
       </c>
       <c r="E42" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F42" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="G42" t="n">
         <v>17</v>
@@ -8046,146 +8044,148 @@
         <v>0</v>
       </c>
       <c r="I42" t="n">
-        <v>592.2</v>
+        <v>126.87</v>
       </c>
       <c r="J42" t="n">
-        <v>593.39</v>
+        <v>105.19</v>
       </c>
       <c r="K42" t="n">
-        <v>-0.2</v>
+        <v>20.6</v>
       </c>
       <c r="L42" t="n">
-        <v>74.02</v>
+        <v>67.15000000000001</v>
       </c>
       <c r="M42" t="n">
-        <v>0.21</v>
+        <v>2.63</v>
       </c>
       <c r="N42" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>07-09-2026</t>
+          <t>25-06-2026</t>
         </is>
       </c>
       <c r="P42" t="n">
-        <v>0.022</v>
+        <v>0.052</v>
       </c>
       <c r="Q42" t="n">
-        <v>941</v>
-      </c>
-      <c r="R42" t="inlineStr"/>
+        <v>5034</v>
+      </c>
+      <c r="R42" t="n">
+        <v>32.8</v>
+      </c>
       <c r="S42" t="n">
-        <v>-2</v>
+        <v>-25</v>
       </c>
       <c r="T42" t="n">
-        <v>5</v>
+        <v>71</v>
       </c>
       <c r="U42" t="n">
-        <v>-152</v>
+        <v>-11</v>
       </c>
       <c r="V42" t="n">
-        <v>-6.5</v>
+        <v>1.48</v>
       </c>
       <c r="W42" t="n">
-        <v>9.24</v>
+        <v>10.7</v>
       </c>
       <c r="X42" t="n">
-        <v>2.23</v>
+        <v>0</v>
       </c>
       <c r="Y42" t="b">
         <v>1</v>
       </c>
       <c r="Z42" t="n">
-        <v>6</v>
+        <v>69</v>
       </c>
       <c r="AA42" t="n">
-        <v>590.46</v>
+        <v>109.5</v>
       </c>
       <c r="AB42" t="n">
-        <v>545.01</v>
+        <v>112.05</v>
       </c>
       <c r="AC42" t="n">
-        <v>17.9</v>
+        <v>27.3</v>
       </c>
       <c r="AD42" t="n">
-        <v>593.3866666666667</v>
+        <v>105.19</v>
       </c>
       <c r="AE42" t="n">
-        <v>-0.2</v>
+        <v>20.6</v>
       </c>
       <c r="AF42" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Stale</t>
         </is>
       </c>
       <c r="AG42" t="inlineStr">
         <is>
-          <t>Confirmed Accumulation</t>
+          <t>Stale Accumulation</t>
         </is>
       </c>
       <c r="AH42" t="inlineStr">
         <is>
-          <t>Confirmed Accumulation</t>
+          <t>Late — Poor Entry</t>
         </is>
       </c>
       <c r="AI42" t="inlineStr">
         <is>
-          <t>28-08-2026</t>
+          <t>25-06-2026</t>
         </is>
       </c>
       <c r="AJ42" t="inlineStr">
         <is>
-          <t>07-09-2026</t>
+          <t>25-06-2026</t>
         </is>
       </c>
       <c r="AK42" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="AL42" t="n">
-        <v>18</v>
+        <v>82</v>
       </c>
       <c r="AM42" t="n">
-        <v>8</v>
+        <v>82</v>
       </c>
       <c r="AN42" t="n">
         <v>0</v>
       </c>
       <c r="AO42" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AP42" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AQ42" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AR42" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AS42" t="n">
         <v>0</v>
       </c>
       <c r="AT42" t="n">
-        <v>966192</v>
+        <v>0</v>
       </c>
       <c r="AU42" t="n">
-        <v>2136192</v>
+        <v>0</v>
       </c>
       <c r="AV42" t="n">
-        <v>2136192</v>
+        <v>0</v>
       </c>
       <c r="AW42" t="n">
-        <v>2136192</v>
+        <v>78892500</v>
       </c>
       <c r="AX42" t="n">
         <v>0</v>
       </c>
       <c r="AY42" t="n">
-        <v>2136192</v>
+        <v>0</v>
       </c>
       <c r="AZ42" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="BA42" t="n">
         <v>0</v>
@@ -8249,13 +8249,13 @@
         </is>
       </c>
       <c r="P43" t="n">
-        <v>2.271</v>
+        <v>2.27</v>
       </c>
       <c r="Q43" t="n">
-        <v>24551</v>
+        <v>24554</v>
       </c>
       <c r="R43" t="n">
-        <v>31</v>
+        <v>31.1</v>
       </c>
       <c r="S43" t="n">
         <v>-2</v>
@@ -8431,13 +8431,13 @@
         </is>
       </c>
       <c r="P44" t="n">
-        <v>0.166</v>
+        <v>0.169</v>
       </c>
       <c r="Q44" t="n">
-        <v>745</v>
+        <v>735</v>
       </c>
       <c r="R44" t="n">
-        <v>13.6</v>
+        <v>13.4</v>
       </c>
       <c r="S44" t="n">
         <v>185</v>
@@ -8793,10 +8793,10 @@
         </is>
       </c>
       <c r="P46" t="n">
-        <v>0.127</v>
+        <v>0.128</v>
       </c>
       <c r="Q46" t="n">
-        <v>583</v>
+        <v>580</v>
       </c>
       <c r="R46" t="n">
         <v>13.8</v>
@@ -8973,13 +8973,13 @@
         </is>
       </c>
       <c r="P47" t="n">
-        <v>0.04</v>
+        <v>0.041</v>
       </c>
       <c r="Q47" t="n">
-        <v>768</v>
+        <v>755</v>
       </c>
       <c r="R47" t="n">
-        <v>50.1</v>
+        <v>49.2</v>
       </c>
       <c r="S47" t="n">
         <v>7</v>
@@ -9158,10 +9158,10 @@
         <v>0.035</v>
       </c>
       <c r="Q48" t="n">
-        <v>3093</v>
+        <v>3091</v>
       </c>
       <c r="R48" t="n">
-        <v>21</v>
+        <v>20.9</v>
       </c>
       <c r="S48" t="n">
         <v>17</v>
@@ -9337,13 +9337,13 @@
         </is>
       </c>
       <c r="P49" t="n">
-        <v>0.191</v>
+        <v>0.194</v>
       </c>
       <c r="Q49" t="n">
-        <v>470</v>
+        <v>464</v>
       </c>
       <c r="R49" t="n">
-        <v>11.7</v>
+        <v>11.6</v>
       </c>
       <c r="S49" t="n">
         <v>19</v>
@@ -9519,10 +9519,10 @@
         </is>
       </c>
       <c r="P50" t="n">
-        <v>0.29</v>
+        <v>0.289</v>
       </c>
       <c r="Q50" t="n">
-        <v>3529</v>
+        <v>3533</v>
       </c>
       <c r="R50" t="n">
         <v>24.7</v>
@@ -9704,10 +9704,10 @@
         <v>0.052</v>
       </c>
       <c r="Q51" t="n">
-        <v>9076</v>
+        <v>9008</v>
       </c>
       <c r="R51" t="n">
-        <v>15.4</v>
+        <v>15.3</v>
       </c>
       <c r="S51" t="n">
         <v>21</v>
@@ -9886,10 +9886,10 @@
         <v>0.008</v>
       </c>
       <c r="Q52" t="n">
-        <v>112322</v>
+        <v>112251</v>
       </c>
       <c r="R52" t="n">
-        <v>32.4</v>
+        <v>32.3</v>
       </c>
       <c r="S52" t="n">
         <v>18</v>
@@ -10065,13 +10065,13 @@
         </is>
       </c>
       <c r="P53" t="n">
-        <v>0.248</v>
+        <v>0.244</v>
       </c>
       <c r="Q53" t="n">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="R53" t="n">
-        <v>14.9</v>
+        <v>15.1</v>
       </c>
       <c r="S53" t="n">
         <v>16</v>
@@ -10247,13 +10247,13 @@
         </is>
       </c>
       <c r="P54" t="n">
-        <v>0.376</v>
+        <v>0.377</v>
       </c>
       <c r="Q54" t="n">
-        <v>1738</v>
+        <v>1730</v>
       </c>
       <c r="R54" t="n">
-        <v>31.4</v>
+        <v>31.3</v>
       </c>
       <c r="S54" t="n">
         <v>39</v>
@@ -10429,13 +10429,13 @@
         </is>
       </c>
       <c r="P55" t="n">
-        <v>0.042</v>
+        <v>0.041</v>
       </c>
       <c r="Q55" t="n">
-        <v>1486</v>
+        <v>1500</v>
       </c>
       <c r="R55" t="n">
-        <v>18.8</v>
+        <v>19</v>
       </c>
       <c r="S55" t="n">
         <v>13</v>
@@ -10611,13 +10611,13 @@
         </is>
       </c>
       <c r="P56" t="n">
-        <v>0.052</v>
+        <v>0.05</v>
       </c>
       <c r="Q56" t="n">
-        <v>907</v>
+        <v>935</v>
       </c>
       <c r="R56" t="n">
-        <v>24.7</v>
+        <v>25.5</v>
       </c>
       <c r="S56" t="n">
         <v>9</v>
@@ -11518,7 +11518,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>PNGS REVA DIAMOND JEWELLERY LIMITED</t>
+          <t>PNGS Reva Diamond Jewellery Limited</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -12073,105 +12073,105 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>TAINWALCHM</t>
+          <t>SGIL</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>TAINWALA CHEMICALS AND PLASTICS (INDIA) LIMITED</t>
+          <t>SYNERGY GREEN INDUSTRIES LIMITED</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>207.79</v>
+        <v>592.2</v>
       </c>
       <c r="D38" t="n">
-        <v>210.84</v>
+        <v>593.62</v>
       </c>
       <c r="E38" t="n">
-        <v>-1.4</v>
+        <v>-0.2</v>
       </c>
       <c r="F38" t="n">
-        <v>67.04000000000001</v>
+        <v>74.02</v>
       </c>
       <c r="G38" t="n">
-        <v>0.42</v>
+        <v>0.25</v>
       </c>
       <c r="H38" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>10-09-2026</t>
+          <t>11-09-2026</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>HCLTECH</t>
+          <t>TAINWALCHM</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>HCL Technologies Limited</t>
+          <t>TAINWALA CHEMICALS AND PLASTICS (INDIA) LIMITED</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>1206.1</v>
+        <v>207.79</v>
       </c>
       <c r="D39" t="n">
-        <v>1104.34</v>
+        <v>210.84</v>
       </c>
       <c r="E39" t="n">
-        <v>9.199999999999999</v>
+        <v>-1.4</v>
       </c>
       <c r="F39" t="n">
-        <v>60.82</v>
+        <v>67.04000000000001</v>
       </c>
       <c r="G39" t="n">
-        <v>5.22</v>
+        <v>0.42</v>
       </c>
       <c r="H39" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>12-06-2026</t>
+          <t>10-09-2026</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>MANINFRA</t>
+          <t>HCLTECH</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>MAN INFRACONSTRUCTION LIMITED</t>
+          <t>HCL Technologies Limited</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>126.87</v>
+        <v>1206.1</v>
       </c>
       <c r="D40" t="n">
-        <v>105.19</v>
+        <v>1104.34</v>
       </c>
       <c r="E40" t="n">
-        <v>20.6</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="F40" t="n">
-        <v>67.15000000000001</v>
+        <v>60.82</v>
       </c>
       <c r="G40" t="n">
-        <v>2.63</v>
+        <v>5.22</v>
       </c>
       <c r="H40" t="n">
         <v>1</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>25-06-2026</t>
+          <t>12-06-2026</t>
         </is>
       </c>
     </row>
@@ -12213,35 +12213,35 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>SGIL</t>
+          <t>MANINFRA</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>SYNERGY GREEN INDUSTRIES LIMITED</t>
+          <t>MAN INFRACONSTRUCTION LIMITED</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>592.2</v>
+        <v>126.87</v>
       </c>
       <c r="D42" t="n">
-        <v>593.39</v>
+        <v>105.19</v>
       </c>
       <c r="E42" t="n">
-        <v>-0.2</v>
+        <v>20.6</v>
       </c>
       <c r="F42" t="n">
-        <v>74.02</v>
+        <v>67.15000000000001</v>
       </c>
       <c r="G42" t="n">
-        <v>0.21</v>
+        <v>2.63</v>
       </c>
       <c r="H42" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>07-09-2026</t>
+          <t>25-06-2026</t>
         </is>
       </c>
     </row>
@@ -12818,7 +12818,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8">
@@ -12838,7 +12838,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10">

</xml_diff>